<commit_message>
15/06/2023 time 5.55 PM
</commit_message>
<xml_diff>
--- a/E-commerce/Data/TestData.xlsx
+++ b/E-commerce/Data/TestData.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26501"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{B925C988-17CD-4C75-BA71-6174C34B7984}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{E864D2A3-116B-49D3-82AA-D65EC7366496}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="92">
   <si>
     <t>username</t>
   </si>
@@ -192,6 +192,114 @@
   </si>
   <si>
     <t>America</t>
+  </si>
+  <si>
+    <t>Blood Type</t>
+  </si>
+  <si>
+    <t>A+</t>
+  </si>
+  <si>
+    <t>A-</t>
+  </si>
+  <si>
+    <t>B+</t>
+  </si>
+  <si>
+    <t>B-</t>
+  </si>
+  <si>
+    <t>O+</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>99</t>
+  </si>
+  <si>
+    <t>98</t>
+  </si>
+  <si>
+    <t>97</t>
+  </si>
+  <si>
+    <t>96</t>
+  </si>
+  <si>
+    <t>95</t>
+  </si>
+  <si>
+    <t>11111</t>
+  </si>
+  <si>
+    <t>22222</t>
+  </si>
+  <si>
+    <t>33333</t>
+  </si>
+  <si>
+    <t>44444</t>
+  </si>
+  <si>
+    <t>55555</t>
+  </si>
+  <si>
+    <t>45086</t>
+  </si>
+  <si>
+    <t>45453</t>
+  </si>
+  <si>
+    <t>45819</t>
+  </si>
+  <si>
+    <t>46185</t>
+  </si>
+  <si>
+    <t>46551</t>
+  </si>
+  <si>
+    <t>5555</t>
+  </si>
+  <si>
+    <t>4444</t>
+  </si>
+  <si>
+    <t>3333</t>
+  </si>
+  <si>
+    <t>2222</t>
+  </si>
+  <si>
+    <t>1111</t>
+  </si>
+  <si>
+    <t>45087</t>
+  </si>
+  <si>
+    <t>45088</t>
+  </si>
+  <si>
+    <t>45089</t>
+  </si>
+  <si>
+    <t>45090</t>
+  </si>
+  <si>
+    <t>Female</t>
   </si>
 </sst>
 </file>
@@ -294,7 +402,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
@@ -317,6 +425,9 @@
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -808,13 +919,19 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{540B3813-FEF7-4622-BA72-342EAA1B5206}">
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16384" width="8.88671875" style="11"/>
+    <col min="1" max="3" width="8.88671875" style="11"/>
+    <col min="4" max="4" width="11.5546875" style="11" customWidth="1"/>
+    <col min="5" max="5" width="11" style="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="10" width="8.88671875" style="11"/>
+    <col min="11" max="11" width="10.44140625" style="11" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13" style="11" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="8.88671875" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>13</v>
       </c>
@@ -860,8 +977,11 @@
       <c r="O1" s="9" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P1" s="12" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>16</v>
       </c>
@@ -874,23 +994,23 @@
       <c r="D2" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="10">
-        <v>1</v>
-      </c>
-      <c r="F2" s="10">
-        <v>99</v>
-      </c>
-      <c r="G2" s="10">
-        <v>11111</v>
-      </c>
-      <c r="H2" s="10">
-        <v>45086</v>
-      </c>
-      <c r="I2" s="10">
-        <v>11111</v>
-      </c>
-      <c r="J2" s="10">
-        <v>5555</v>
+      <c r="E2" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="J2" s="10" t="s">
+        <v>82</v>
       </c>
       <c r="K2" s="10" t="s">
         <v>41</v>
@@ -904,11 +1024,14 @@
       <c r="N2" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="O2" s="10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="O2" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="P2" s="10" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>19</v>
       </c>
@@ -921,23 +1044,23 @@
       <c r="D3" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="E3" s="10">
-        <v>2</v>
-      </c>
-      <c r="F3" s="10">
-        <v>98</v>
-      </c>
-      <c r="G3" s="10">
-        <v>22222</v>
-      </c>
-      <c r="H3" s="10">
-        <v>45453</v>
-      </c>
-      <c r="I3" s="10">
-        <v>22222</v>
-      </c>
-      <c r="J3" s="10">
-        <v>4444</v>
+      <c r="E3" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="I3" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="J3" s="10" t="s">
+        <v>83</v>
       </c>
       <c r="K3" s="10" t="s">
         <v>46</v>
@@ -945,17 +1068,20 @@
       <c r="L3" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="M3" s="10">
-        <v>45087</v>
+      <c r="M3" s="10" t="s">
+        <v>87</v>
       </c>
       <c r="N3" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="O3" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+      <c r="O3" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="P3" s="10" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
         <v>22</v>
       </c>
@@ -968,23 +1094,23 @@
       <c r="D4" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="E4" s="10">
-        <v>3</v>
-      </c>
-      <c r="F4" s="10">
-        <v>97</v>
-      </c>
-      <c r="G4" s="10">
-        <v>33333</v>
-      </c>
-      <c r="H4" s="10">
-        <v>45819</v>
-      </c>
-      <c r="I4" s="10">
-        <v>33333</v>
-      </c>
-      <c r="J4" s="10">
-        <v>3333</v>
+      <c r="E4" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>84</v>
       </c>
       <c r="K4" s="10" t="s">
         <v>48</v>
@@ -992,17 +1118,20 @@
       <c r="L4" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="M4" s="10">
-        <v>45088</v>
+      <c r="M4" s="10" t="s">
+        <v>88</v>
       </c>
       <c r="N4" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="O4" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="O4" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="P4" s="10" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
         <v>25</v>
       </c>
@@ -1015,23 +1144,23 @@
       <c r="D5" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="E5" s="10">
-        <v>4</v>
-      </c>
-      <c r="F5" s="10">
-        <v>96</v>
-      </c>
-      <c r="G5" s="10">
-        <v>44444</v>
-      </c>
-      <c r="H5" s="10">
-        <v>46185</v>
-      </c>
-      <c r="I5" s="10">
-        <v>44444</v>
-      </c>
-      <c r="J5" s="10">
-        <v>2222</v>
+      <c r="E5" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="J5" s="10" t="s">
+        <v>85</v>
       </c>
       <c r="K5" s="10" t="s">
         <v>50</v>
@@ -1039,17 +1168,20 @@
       <c r="L5" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="M5" s="10">
-        <v>45089</v>
+      <c r="M5" s="10" t="s">
+        <v>89</v>
       </c>
       <c r="N5" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="O5" s="10">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="O5" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="P5" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
         <v>51</v>
       </c>
@@ -1062,23 +1194,23 @@
       <c r="D6" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="E6" s="10">
-        <v>5</v>
-      </c>
-      <c r="F6" s="10">
-        <v>95</v>
-      </c>
-      <c r="G6" s="10">
-        <v>55555</v>
-      </c>
-      <c r="H6" s="10">
-        <v>46551</v>
-      </c>
-      <c r="I6" s="10">
-        <v>55555</v>
-      </c>
-      <c r="J6" s="10">
-        <v>1111</v>
+      <c r="E6" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="J6" s="10" t="s">
+        <v>86</v>
       </c>
       <c r="K6" s="10" t="s">
         <v>55</v>
@@ -1086,14 +1218,17 @@
       <c r="L6" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="M6" s="10">
-        <v>45090</v>
+      <c r="M6" s="10" t="s">
+        <v>90</v>
       </c>
       <c r="N6" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="O6" s="10">
-        <v>5</v>
+        <v>91</v>
+      </c>
+      <c r="O6" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="P6" s="10" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update by maruti kolavale 19-march -2026
</commit_message>
<xml_diff>
--- a/E-commerce/Data/TestData.xlsx
+++ b/E-commerce/Data/TestData.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{0DEB02C5-A3F5-4E3B-BEA3-D7A51BDC812F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{9C11308A-F281-4F34-8676-8B7778D032C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="72" yWindow="0" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Validcreads" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
     <sheet name="Sheet3" sheetId="7" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:Q10"/>
+  <oleSize ref="A1:N10"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>